<commit_message>
docs(inspeccion): correccion Anexo A - preparacion individual (Inspector 2)
</commit_message>
<xml_diff>
--- a/02_Inspeccion/AnexoA_checklists/AnexoA_checklist_Inspector2_Mayra_Cordova.xlsx
+++ b/02_Inspeccion/AnexoA_checklists/AnexoA_checklist_Inspector2_Mayra_Cordova.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy Mendoza\Desktop\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F5B0FEA-C76A-4F5A-BE28-815B1D7BD883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D208857-6051-4A01-B5B8-6E72B4A11274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -284,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -297,79 +297,32 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -761,24 +714,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -818,7 +771,7 @@
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" t="s">
         <v>49</v>
       </c>
     </row>
@@ -826,7 +779,7 @@
       <c r="D7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" t="s">
         <v>50</v>
       </c>
     </row>
@@ -836,14 +789,14 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
@@ -875,13 +828,13 @@
       <c r="C12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="9" t="s">
         <v>38</v>
       </c>
     </row>
@@ -893,13 +846,13 @@
         <v>21</v>
       </c>
       <c r="C13" s="6"/>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="9" t="s">
         <v>40</v>
       </c>
     </row>
@@ -913,13 +866,13 @@
       <c r="C14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="9" t="s">
         <v>42</v>
       </c>
     </row>
@@ -931,13 +884,13 @@
         <v>23</v>
       </c>
       <c r="C15" s="6"/>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="F15" s="9" t="s">
         <v>44</v>
       </c>
     </row>
@@ -951,13 +904,13 @@
       <c r="C16" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="9" t="s">
         <v>46</v>
       </c>
     </row>
@@ -969,13 +922,13 @@
         <v>25</v>
       </c>
       <c r="C17" s="6"/>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="29" t="s">
+      <c r="E17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="31" t="s">
+      <c r="F17" s="9" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1058,30 +1011,32 @@
       <c r="F23" s="7"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="32"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="19">
+        <v>6</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="35">
+      <c r="B28" s="14">
         <v>46242</v>
       </c>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>